<commit_message>
Neutralize dataset source wording
</commit_message>
<xml_diff>
--- a/outputs/executive_dashboard.xlsx
+++ b/outputs/executive_dashboard.xlsx
@@ -573,7 +573,7 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -610,7 +610,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -626,14 +626,14 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -649,14 +649,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Core samples emphasize quality; extended samples exercise scale and task taxonomy.</t>
+          <t>Core samples emphasize quality; extended samples exercise scale and task coverage.</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -6345,7 +6345,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -6905,7 +6905,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>reference_style_extended</t>
+          <t>extended_diagnostic_45</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">

</xml_diff>